<commit_message>
fix(grove): same-day aToken events dropped from cumulative — Grove April profit +$1.41M (#133)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-04/grove_settlement_april_2026.xlsx
+++ b/settlements/grove/2026-04/grove_settlement_april_2026.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>5210896.698222283</v>
+        <v>6622808.993949268</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>5256229.526710057</v>
+        <v>6668141.822437041</v>
       </c>
     </row>
     <row r="8">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>5210896.698222283</v>
+        <v>6622808.993949268</v>
       </c>
     </row>
     <row r="20">
@@ -618,7 +618,7 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>2270604.88273054</v>
+        <v>3682517.178457524</v>
       </c>
     </row>
     <row r="23">
@@ -653,7 +653,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-10T10:52:07+00:00</t>
+          <t>2026-06-10T15:01:23+00:00</t>
         </is>
       </c>
     </row>
@@ -988,13 +988,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>798983.3608645581</v>
+        <v>798332.6224423209</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>798983.3608645581</v>
+        <v>798332.6224423209</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>383782.3196085766</v>
+        <v>384433.0580308138</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1047,19 +1047,19 @@
         <v>0</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>164994117.6754281</v>
+        <v>166094117.6754281</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>513190.3775715641</v>
+        <v>516191.0101208151</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>513190.3775715641</v>
+        <v>516191.0101208151</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>625594.5730965375</v>
+        <v>622593.9405472864</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1118,13 +1118,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>398874.9083768068</v>
+        <v>398550.0415006478</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>398874.9083768068</v>
+        <v>398550.0415006478</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>191594.9005557068</v>
+        <v>191919.7674318658</v>
       </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
@@ -1183,13 +1183,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>313936.2460300053</v>
+        <v>313680.5581303178</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>313936.2460300053</v>
+        <v>313680.5581303178</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>260344.8539699948</v>
+        <v>260600.5418696821</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1230,31 +1230,31 @@
         <v>-138267796.0572637</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-1348288.147999676</v>
+        <v>63624.14772730789</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>1411897.309885636</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>63609.1618859599</v>
+        <v>1475521.457612944</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>77820296.86848758</v>
+        <v>77490850.66615129</v>
       </c>
       <c r="M8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>242048.7960136409</v>
+        <v>240827.7971568373</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>242048.7960136409</v>
+        <v>240827.7971568373</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-178439.6341276809</v>
+        <v>1234693.660456107</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1313,13 +1313,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>157616.5478947693</v>
+        <v>157488.1758300688</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>157616.5478947693</v>
+        <v>157488.1758300688</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>33437.81041663571</v>
+        <v>33566.1824813362</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1378,13 +1378,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>155517.7799068868</v>
+        <v>155391.1172006485</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>155517.7799068868</v>
+        <v>155391.1172006485</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>247225.1800931131</v>
+        <v>247351.8427993514</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1447,13 +1447,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>127141.9325754838</v>
+        <v>127038.3808062519</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>127141.9325754838</v>
+        <v>127038.3808062519</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>9752.371987611881</v>
+        <v>9855.923756843762</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1512,13 +1512,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>77806.42400195355</v>
+        <v>77743.05393434642</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>77806.42400195355</v>
+        <v>77743.05393434642</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-67140.86883795355</v>
+        <v>-67077.49877034643</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1577,13 +1577,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>77761.81041589502</v>
+        <v>77698.47668418176</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>77761.81041589502</v>
+        <v>77698.47668418176</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>-77536.6530996597</v>
+        <v>-77473.31936794645</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1642,13 +1642,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>62681.03919654229</v>
+        <v>62629.98812020096</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>62681.03919654229</v>
+        <v>62629.98812020096</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-12826.36091734772</v>
+        <v>-12775.30984100639</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1707,13 +1707,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>9701.788589956248</v>
+        <v>9693.886890234897</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>9701.788589956248</v>
+        <v>9693.886890234897</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>-1181.339322911833</v>
+        <v>-1173.437623190483</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1772,13 +1772,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>3133.389072598707</v>
+        <v>3130.837058675474</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>3133.389072598707</v>
+        <v>3130.837058675474</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>311.1442890097251</v>
+        <v>313.6963029329585</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>1866.096876358804</v>
+        <v>1864.577018754073</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>1866.096876358804</v>
+        <v>1864.577018754073</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-1866.096876368241</v>
+        <v>-1864.57701876351</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1902,13 +1902,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>31.31810472118654</v>
+        <v>31.29259743899273</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>31.31810472118654</v>
+        <v>31.29259743899273</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>-31.31810472118654</v>
+        <v>-31.29259743899273</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1967,13 +1967,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>3.110355598137735e-09</v>
+        <v>3.10782234401297e-09</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>3.110355598137735e-09</v>
+        <v>3.10782234401297e-09</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-3.110355598137735e-09</v>
+        <v>-3.10782234401297e-09</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(grove): Chronicle VAO Router migration — frozen ACRDX feed, Apr–Jul restated (+$144K) (#172)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-04/grove_settlement_april_2026.xlsx
+++ b/settlements/grove/2026-04/grove_settlement_april_2026.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6622808.993949277</v>
+        <v>6540434.835030718</v>
       </c>
     </row>
     <row r="5">
@@ -515,168 +515,178 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>6793231.992437051</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>+ chronicle_points (20% of base rate on Chronicle Farm USDS)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>17001.12794103559</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" s="4" t="n">
+        <v>6727858.961459527</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>2946944.561473255</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2946944.561473255</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>6395006.500245043</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="n">
         <v>9341951.061718298</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Sky Revenue (max) — BR × full ilk debt, no deductions</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CoF on Net_Subs (actual BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>2946944.561473255</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>CoF on Net_Subs (actual BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>2946944.561473255</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>reduction from idle/SDE deductions</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B17" s="3" t="n">
         <v>-7396515.160294596</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
         <v>10343459.72176785</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>6622808.993949277</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6540434.835030718</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>-2946944.561473255</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" s="4" t="n">
-        <v>3675864.432476022</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-04-01 → 2026-04-30 (30 days)</t>
-        </is>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" s="4" t="n">
+        <v>3593490.273557463</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>avalanche_c=84298393, base=45402126, ethereum=24996367, monad=71616121, plume=65382097</t>
+          <t>2026-04-01 → 2026-04-30 (30 days)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-31T00:11:36+00:00</t>
+          <t>avalanche_c=84298393, base=45402126, ethereum=24996367, monad=71616121, plume=65382097</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-08-06T00:21:56+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
@@ -693,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1302,19 +1312,19 @@
         <v>50674767.8590638</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>50865822.2173752</v>
+        <v>50783448.05845664</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>191054.358311405</v>
+        <v>108680.1993928453</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>191054.358311405</v>
+        <v>108680.1993928453</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>191054.358311405</v>
+        <v>108680.1993928453</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>0</v>
@@ -1332,7 +1342,7 @@
         <v>154754.4628511592</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>36299.89546024581</v>
+        <v>-46074.26345831385</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -2783,59 +2793,189 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>E40</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>USDS raw (Diamond PAU ALM idle)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E41</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JTRSY Basin escrow — USDS pending subscription (Diamond PAU)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="inlineStr">
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
@@ -2928,7 +3068,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Reference rate (tbill_3m), period avg</t>
+          <t>Reference rate (tbill_3m→sofr@2026-07-23), period avg</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">

</xml_diff>